<commit_message>
Fix duplicate DUID rows in summary.csv
eli_per_duid.feather had duplicate MAPS2PV1 and MBPS2PV1 rows, inflating
the left-join in build_summary to 240 rows / 238 unique DUIDs.

- Dedupe the seeded feather (106 → 104 rows)
- drop_duplicates before the merge as a defensive guard
- Assert DUID uniqueness in tests/validate_outputs.py so any future
  regression fails CI instead of shipping phantom rows

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-07
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -532,12 +532,12 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Actual FY23-24</t>
+          <t>Actual FY24-25</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Actual FY24-25</t>
+          <t>Actual FY25-26</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -644,11 +644,9 @@
         <v>132</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.0511</v>
-      </c>
-      <c r="K2" s="5" t="n">
         <v>0.1441</v>
       </c>
+      <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -729,11 +727,9 @@
         <v>66</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.0521</v>
-      </c>
-      <c r="K3" s="5" t="n">
         <v>0.128</v>
       </c>
+      <c r="K3" s="5" t="inlineStr"/>
       <c r="L3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -814,11 +810,9 @@
         <v>132</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="K4" s="5" t="n">
         <v>0.123</v>
       </c>
+      <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -899,11 +893,9 @@
         <v>22</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="K5" s="5" t="n">
         <v>0.1492</v>
       </c>
+      <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -1039,11 +1031,9 @@
         <v>132</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.0327</v>
-      </c>
-      <c r="K7" s="5" t="n">
         <v>0.0292</v>
       </c>
+      <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1108,11 +1098,9 @@
         <v>132</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0862</v>
-      </c>
-      <c r="K8" s="5" t="n">
         <v>0.0799</v>
       </c>
+      <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -1248,11 +1236,9 @@
         <v>132</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="K10" s="5" t="n">
         <v>0.0833</v>
       </c>
+      <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1317,11 +1303,9 @@
         <v>132</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.0643</v>
-      </c>
-      <c r="K11" s="5" t="n">
         <v>0.0762</v>
       </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="n">
         <v>0.7032826997896851</v>
       </c>
@@ -1441,11 +1425,9 @@
         <v>66</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="K13" s="5" t="n">
         <v>0.3285</v>
       </c>
+      <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1591,11 +1573,9 @@
         <v>330</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="K15" s="5" t="n">
         <v>0.1353</v>
       </c>
+      <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -1660,11 +1640,9 @@
         <v>132</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.1268</v>
-      </c>
-      <c r="K16" s="5" t="n">
         <v>0.1778</v>
       </c>
+      <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -1745,11 +1723,9 @@
         <v>132</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.1304</v>
-      </c>
-      <c r="K17" s="5" t="n">
         <v>0.2781</v>
       </c>
+      <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1814,11 +1790,9 @@
         <v>66</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.06950000000000001</v>
-      </c>
-      <c r="K18" s="5" t="n">
         <v>0.1147</v>
       </c>
+      <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1883,11 +1857,9 @@
         <v>132</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.1534</v>
-      </c>
-      <c r="K19" s="5" t="n">
         <v>0.2801</v>
       </c>
+      <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -1968,11 +1940,9 @@
         <v>220</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="K20" s="5" t="n">
         <v>0.2431</v>
       </c>
+      <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2053,11 +2023,9 @@
         <v>22</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="K21" s="5" t="n">
         <v>0.2403</v>
       </c>
+      <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2138,11 +2106,9 @@
         <v>132</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.4514</v>
-      </c>
-      <c r="K22" s="5" t="n">
         <v>0.5511</v>
       </c>
+      <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2223,11 +2189,9 @@
         <v>132</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="K23" s="5" t="n">
         <v>0.0614</v>
       </c>
+      <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2308,11 +2272,9 @@
         <v>66</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="K24" s="5" t="n">
         <v>0.5639</v>
       </c>
+      <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2393,11 +2355,9 @@
         <v>66</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="K25" s="5" t="n">
         <v>0.0089</v>
       </c>
+      <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -2649,11 +2609,9 @@
         <v>132</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.0332</v>
-      </c>
-      <c r="K29" s="5" t="n">
         <v>0.078</v>
       </c>
+      <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2734,11 +2692,9 @@
         <v>330</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0851</v>
-      </c>
-      <c r="K30" s="5" t="n">
         <v>0.125</v>
       </c>
+      <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2819,11 +2775,9 @@
         <v>330</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.0885</v>
-      </c>
-      <c r="K31" s="5" t="n">
         <v>0.1153</v>
       </c>
+      <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2904,11 +2858,9 @@
         <v>132</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0277</v>
-      </c>
-      <c r="K32" s="5" t="n">
         <v>0.0388</v>
       </c>
+      <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2989,11 +2941,9 @@
         <v>66</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="K33" s="5" t="n">
         <v>0.2694</v>
       </c>
+      <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -3168,11 +3118,9 @@
         <v>220</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="K36" s="5" t="n">
         <v>0.1146</v>
       </c>
+      <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -3253,11 +3201,9 @@
         <v>132</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.1766</v>
-      </c>
-      <c r="K37" s="5" t="n">
         <v>0.2365</v>
       </c>
+      <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -3565,11 +3511,9 @@
         <v>132</v>
       </c>
       <c r="J41" s="5" t="n">
-        <v>0.1231</v>
-      </c>
-      <c r="K41" s="5" t="n">
         <v>0.1167</v>
       </c>
+      <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3650,11 +3594,9 @@
         <v>66</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.1585</v>
-      </c>
-      <c r="K42" s="5" t="n">
         <v>0.2501</v>
       </c>
+      <c r="K42" s="5" t="inlineStr"/>
       <c r="L42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3864,10 +3806,10 @@
       <c r="I45" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="J45" s="5" t="inlineStr"/>
-      <c r="K45" s="5" t="n">
+      <c r="J45" s="5" t="n">
         <v>0.0616</v>
       </c>
+      <c r="K45" s="5" t="inlineStr"/>
       <c r="L45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3948,11 +3890,9 @@
         <v>132</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>0.0315</v>
-      </c>
-      <c r="K46" s="5" t="n">
         <v>0.0306</v>
       </c>
+      <c r="K46" s="5" t="inlineStr"/>
       <c r="L46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -4033,11 +3973,9 @@
         <v>132</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>0.1433</v>
-      </c>
-      <c r="K47" s="5" t="n">
         <v>0.1883</v>
       </c>
+      <c r="K47" s="5" t="inlineStr"/>
       <c r="L47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -4102,11 +4040,9 @@
         <v>132</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>0.06519999999999999</v>
-      </c>
-      <c r="K48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
+      <c r="K48" s="5" t="inlineStr"/>
       <c r="L48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -4252,11 +4188,9 @@
         <v>132</v>
       </c>
       <c r="J50" s="5" t="n">
-        <v>0.2031</v>
-      </c>
-      <c r="K50" s="5" t="n">
         <v>0.1969</v>
       </c>
+      <c r="K50" s="5" t="inlineStr"/>
       <c r="L50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -4315,11 +4249,9 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="5" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="K51" s="5" t="n">
         <v>0.0528</v>
       </c>
+      <c r="K51" s="5" t="inlineStr"/>
       <c r="L51" s="5" t="inlineStr"/>
       <c r="M51" s="5" t="inlineStr"/>
       <c r="N51" s="5" t="n">
@@ -4374,11 +4306,9 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="5" t="n">
-        <v>0.0983</v>
-      </c>
-      <c r="K52" s="5" t="n">
         <v>0.1308</v>
       </c>
+      <c r="K52" s="5" t="inlineStr"/>
       <c r="L52" s="5" t="inlineStr"/>
       <c r="M52" s="5" t="inlineStr"/>
       <c r="N52" s="5" t="n">
@@ -4433,11 +4363,9 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="5" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="K53" s="5" t="n">
         <v>0.0143</v>
       </c>
+      <c r="K53" s="5" t="inlineStr"/>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr"/>
       <c r="N53" s="5" t="n">
@@ -4492,11 +4420,9 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="5" t="n">
-        <v>0.0213</v>
-      </c>
-      <c r="K54" s="5" t="n">
         <v>0.0265</v>
       </c>
+      <c r="K54" s="5" t="inlineStr"/>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
       <c r="N54" s="5" t="n">
@@ -4606,11 +4532,9 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="5" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="K56" s="5" t="n">
         <v>0.0066</v>
       </c>
+      <c r="K56" s="5" t="inlineStr"/>
       <c r="L56" s="5" t="inlineStr"/>
       <c r="M56" s="5" t="inlineStr"/>
       <c r="N56" s="5" t="n">
@@ -4775,11 +4699,9 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="5" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="K59" s="5" t="n">
         <v>0.0298</v>
       </c>
+      <c r="K59" s="5" t="inlineStr"/>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
       <c r="N59" s="5" t="n">
@@ -4888,10 +4810,10 @@
         <v>145</v>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="5" t="inlineStr"/>
-      <c r="K61" s="5" t="n">
+      <c r="J61" s="5" t="n">
         <v>0.0509</v>
       </c>
+      <c r="K61" s="5" t="inlineStr"/>
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
       <c r="N61" s="5" t="n">
@@ -4946,11 +4868,9 @@
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="5" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="K62" s="5" t="n">
         <v>0.0168</v>
       </c>
+      <c r="K62" s="5" t="inlineStr"/>
       <c r="L62" s="5" t="inlineStr"/>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="n">
@@ -5005,11 +4925,9 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="5" t="n">
-        <v>0.0155</v>
-      </c>
-      <c r="K63" s="5" t="n">
         <v>0.055</v>
       </c>
+      <c r="K63" s="5" t="inlineStr"/>
       <c r="L63" s="5" t="inlineStr"/>
       <c r="M63" s="5" t="inlineStr"/>
       <c r="N63" s="5" t="n">
@@ -5064,11 +4982,9 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="5" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K64" s="5" t="n">
         <v>0.0178</v>
       </c>
+      <c r="K64" s="5" t="inlineStr"/>
       <c r="L64" s="5" t="inlineStr"/>
       <c r="M64" s="5" t="inlineStr"/>
       <c r="N64" s="5" t="n">
@@ -5122,10 +5038,10 @@
         <v>396</v>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="5" t="inlineStr"/>
-      <c r="K65" s="5" t="n">
+      <c r="J65" s="5" t="n">
         <v>0.0134</v>
       </c>
+      <c r="K65" s="5" t="inlineStr"/>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
       <c r="N65" s="5" t="n">
@@ -5180,11 +5096,9 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="5" t="n">
-        <v>0.0048</v>
-      </c>
-      <c r="K66" s="5" t="n">
         <v>0.0056</v>
       </c>
+      <c r="K66" s="5" t="inlineStr"/>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
       <c r="N66" s="5" t="n">
@@ -5239,11 +5153,9 @@
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="5" t="n">
-        <v>0.0354</v>
-      </c>
-      <c r="K67" s="5" t="n">
         <v>0.064</v>
       </c>
+      <c r="K67" s="5" t="inlineStr"/>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
       <c r="N67" s="5" t="n">
@@ -5298,11 +5210,9 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="K68" s="5" t="n">
         <v>0.0002</v>
       </c>
+      <c r="K68" s="5" t="inlineStr"/>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
       <c r="N68" s="5" t="n">
@@ -5357,11 +5267,9 @@
       </c>
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="5" t="n">
-        <v>0.0291</v>
-      </c>
-      <c r="K69" s="5" t="n">
         <v>0.0573</v>
       </c>
+      <c r="K69" s="5" t="inlineStr"/>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
       <c r="N69" s="5" t="n">
@@ -5416,11 +5324,9 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="5" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="K70" s="5" t="n">
         <v>0.0294</v>
       </c>
+      <c r="K70" s="5" t="inlineStr"/>
       <c r="L70" s="5" t="inlineStr"/>
       <c r="M70" s="5" t="inlineStr"/>
       <c r="N70" s="5" t="n">
@@ -5499,12 +5405,12 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY23-24</t>
+          <t>CURTAILMENT_ACTUAL_FY24-25</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY24-25</t>
+          <t>CURTAILMENT_ACTUAL_FY25-26</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
@@ -5606,11 +5512,9 @@
         <v>0.8395</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.0511</v>
-      </c>
-      <c r="F2" s="5" t="n">
         <v>0.1441</v>
       </c>
+      <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5690,11 +5594,9 @@
         <v>0.9245</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.0521</v>
-      </c>
-      <c r="F3" s="5" t="n">
         <v>0.128</v>
       </c>
+      <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -5774,11 +5676,9 @@
         <v>0.8823</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="F4" s="5" t="n">
         <v>0.123</v>
       </c>
+      <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5858,11 +5758,9 @@
         <v>0.8436</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="F5" s="5" t="n">
         <v>0.1492</v>
       </c>
+      <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -6002,11 +5900,9 @@
         <v>0.8416</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.0327</v>
-      </c>
-      <c r="F7" s="5" t="n">
         <v>0.0292</v>
       </c>
+      <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6070,11 +5966,9 @@
         <v>0.8899</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0862</v>
-      </c>
-      <c r="F8" s="5" t="n">
         <v>0.0799</v>
       </c>
+      <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -6214,11 +6108,9 @@
         <v>0.8554</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="F10" s="5" t="n">
         <v>0.0833</v>
       </c>
+      <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6282,11 +6174,9 @@
         <v>0.8521</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.0643</v>
-      </c>
-      <c r="F11" s="5" t="n">
         <v>0.0762</v>
       </c>
+      <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="n">
         <v>0.7032826997896851</v>
       </c>
@@ -6410,11 +6300,9 @@
         <v>0.8918</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="F13" s="5" t="n">
         <v>0.3285</v>
       </c>
+      <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6558,11 +6446,9 @@
         <v>0.9635</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="F15" s="5" t="n">
         <v>0.1353</v>
       </c>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -6626,11 +6512,9 @@
         <v>0.8463000000000001</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.1268</v>
-      </c>
-      <c r="F16" s="5" t="n">
         <v>0.1778</v>
       </c>
+      <c r="F16" s="5" t="inlineStr"/>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -6710,11 +6594,9 @@
         <v>0.8652</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.1304</v>
-      </c>
-      <c r="F17" s="5" t="n">
         <v>0.2781</v>
       </c>
+      <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6778,11 +6660,9 @@
         <v>0.8962</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.06950000000000001</v>
-      </c>
-      <c r="F18" s="5" t="n">
         <v>0.1147</v>
       </c>
+      <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6846,11 +6726,9 @@
         <v>0.8865</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.1534</v>
-      </c>
-      <c r="F19" s="5" t="n">
         <v>0.2801</v>
       </c>
+      <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -6930,11 +6808,9 @@
         <v>0.8206</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="F20" s="5" t="n">
         <v>0.2431</v>
       </c>
+      <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -7014,11 +6890,9 @@
         <v>0.8268</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="F21" s="5" t="n">
         <v>0.2403</v>
       </c>
+      <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -7098,11 +6972,9 @@
         <v>0.9482</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.4514</v>
-      </c>
-      <c r="F22" s="5" t="n">
         <v>0.5511</v>
       </c>
+      <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7182,11 +7054,9 @@
         <v>0.8657</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="F23" s="5" t="n">
         <v>0.0614</v>
       </c>
+      <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7266,11 +7136,9 @@
         <v>0.9583</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F24" s="5" t="n">
         <v>0.5639</v>
       </c>
+      <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7350,11 +7218,9 @@
         <v>0.8509</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="F25" s="5" t="n">
         <v>0.0089</v>
       </c>
+      <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -7614,11 +7480,9 @@
         <v>0.9273</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.0332</v>
-      </c>
-      <c r="F29" s="5" t="n">
         <v>0.078</v>
       </c>
+      <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7698,11 +7562,9 @@
         <v>0.8911</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0851</v>
-      </c>
-      <c r="F30" s="5" t="n">
         <v>0.125</v>
       </c>
+      <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7782,11 +7644,9 @@
         <v>0.8911</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.0885</v>
-      </c>
-      <c r="F31" s="5" t="n">
         <v>0.1153</v>
       </c>
+      <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7866,11 +7726,9 @@
         <v>0.9699</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0277</v>
-      </c>
-      <c r="F32" s="5" t="n">
         <v>0.0388</v>
       </c>
+      <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7950,11 +7808,9 @@
         <v>0.8918</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="F33" s="5" t="n">
         <v>0.2694</v>
       </c>
+      <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -8138,11 +7994,9 @@
         <v>0.8218</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="F36" s="5" t="n">
         <v>0.1146</v>
       </c>
+      <c r="F36" s="5" t="inlineStr"/>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -8222,11 +8076,9 @@
         <v>0.8865</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>0.1766</v>
-      </c>
-      <c r="F37" s="5" t="n">
         <v>0.2365</v>
       </c>
+      <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -8530,11 +8382,9 @@
         <v>0.9091</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>0.1231</v>
-      </c>
-      <c r="F41" s="5" t="n">
         <v>0.1167</v>
       </c>
+      <c r="F41" s="5" t="inlineStr"/>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8614,11 +8464,9 @@
         <v>0.8824</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.1585</v>
-      </c>
-      <c r="F42" s="5" t="n">
         <v>0.2501</v>
       </c>
+      <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8825,10 +8673,10 @@
       <c r="D45" s="5" t="n">
         <v>0.9376</v>
       </c>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="n">
+      <c r="E45" s="5" t="n">
         <v>0.0616</v>
       </c>
+      <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8908,11 +8756,9 @@
         <v>0.9273</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>0.0315</v>
-      </c>
-      <c r="F46" s="5" t="n">
         <v>0.0306</v>
       </c>
+      <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8992,11 +8838,9 @@
         <v>0.8865</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>0.1433</v>
-      </c>
-      <c r="F47" s="5" t="n">
         <v>0.1883</v>
       </c>
+      <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -9060,11 +8904,9 @@
         <v>0.8265</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>0.06519999999999999</v>
-      </c>
-      <c r="F48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
+      <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -9208,11 +9050,9 @@
         <v>0.8865</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>0.2031</v>
-      </c>
-      <c r="F50" s="5" t="n">
         <v>0.1969</v>
       </c>
+      <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -9276,11 +9116,9 @@
         <v>0.9254</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="F51" s="5" t="n">
         <v>0.0528</v>
       </c>
+      <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr"/>
@@ -9340,11 +9178,9 @@
         <v>0.9391</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0.0983</v>
-      </c>
-      <c r="F52" s="5" t="n">
         <v>0.1308</v>
       </c>
+      <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
@@ -9404,11 +9240,9 @@
         <v>0.9638</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="F53" s="5" t="n">
         <v>0.0143</v>
       </c>
+      <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr"/>
@@ -9468,11 +9302,9 @@
         <v>0.9545</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>0.0213</v>
-      </c>
-      <c r="F54" s="5" t="n">
         <v>0.0265</v>
       </c>
+      <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
@@ -9592,11 +9424,9 @@
         <v>0.9643</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="F56" s="5" t="n">
         <v>0.0066</v>
       </c>
+      <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
@@ -9776,11 +9606,9 @@
         <v>0.9276</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="F59" s="5" t="n">
         <v>0.0298</v>
       </c>
+      <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="5" t="inlineStr"/>
@@ -9899,10 +9727,10 @@
       <c r="D61" s="5" t="n">
         <v>1.0047</v>
       </c>
-      <c r="E61" s="5" t="inlineStr"/>
-      <c r="F61" s="5" t="n">
+      <c r="E61" s="5" t="n">
         <v>0.0509</v>
       </c>
+      <c r="F61" s="5" t="inlineStr"/>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr"/>
@@ -9962,11 +9790,9 @@
         <v>0.9635</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="F62" s="5" t="n">
         <v>0.0168</v>
       </c>
+      <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr"/>
@@ -10026,11 +9852,9 @@
         <v>0.9635</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>0.0155</v>
-      </c>
-      <c r="F63" s="5" t="n">
         <v>0.055</v>
       </c>
+      <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
       <c r="I63" s="5" t="inlineStr"/>
@@ -10090,11 +9914,9 @@
         <v>0.9528</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="F64" s="5" t="n">
         <v>0.0178</v>
       </c>
+      <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr"/>
@@ -10153,10 +9975,10 @@
       <c r="D65" s="5" t="n">
         <v>0.9618</v>
       </c>
-      <c r="E65" s="5" t="inlineStr"/>
-      <c r="F65" s="5" t="n">
+      <c r="E65" s="5" t="n">
         <v>0.0134</v>
       </c>
+      <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr"/>
@@ -10216,11 +10038,9 @@
         <v>0.8661</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>0.0048</v>
-      </c>
-      <c r="F66" s="5" t="n">
         <v>0.0056</v>
       </c>
+      <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr"/>
@@ -10280,11 +10100,9 @@
         <v>0.896</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>0.0354</v>
-      </c>
-      <c r="F67" s="5" t="n">
         <v>0.064</v>
       </c>
+      <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
       <c r="I67" s="5" t="inlineStr"/>
@@ -10344,11 +10162,9 @@
         <v>1.0029</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="F68" s="5" t="n">
         <v>0.0002</v>
       </c>
+      <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr"/>
@@ -10408,11 +10224,9 @@
         <v>0.8265</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>0.0291</v>
-      </c>
-      <c r="F69" s="5" t="n">
         <v>0.0573</v>
       </c>
+      <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr"/>
@@ -10472,11 +10286,9 @@
         <v>0.9694</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="F70" s="5" t="n">
         <v>0.0294</v>
       </c>
+      <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-08
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -646,7 +646,9 @@
       <c r="J2" s="5" t="n">
         <v>0.1441</v>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="n">
+        <v>0.1695</v>
+      </c>
       <c r="L2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -729,7 +731,9 @@
       <c r="J3" s="5" t="n">
         <v>0.128</v>
       </c>
-      <c r="K3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="n">
+        <v>0.078</v>
+      </c>
       <c r="L3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -812,7 +816,9 @@
       <c r="J4" s="5" t="n">
         <v>0.123</v>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="n">
+        <v>0.1001</v>
+      </c>
       <c r="L4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -895,7 +901,9 @@
       <c r="J5" s="5" t="n">
         <v>0.1492</v>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="n">
+        <v>0.2117</v>
+      </c>
       <c r="L5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -1033,7 +1041,9 @@
       <c r="J7" s="5" t="n">
         <v>0.0292</v>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="n">
+        <v>0.0415</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1100,7 +1110,9 @@
       <c r="J8" s="5" t="n">
         <v>0.0799</v>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="n">
+        <v>0.1689</v>
+      </c>
       <c r="L8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -1175,7 +1187,9 @@
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="n">
+        <v>0.342</v>
+      </c>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
       <c r="N9" s="5" t="n">
@@ -1238,7 +1252,9 @@
       <c r="J10" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="n">
+        <v>0.1175</v>
+      </c>
       <c r="L10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1427,7 +1443,9 @@
       <c r="J13" s="5" t="n">
         <v>0.3285</v>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="n">
+        <v>0.3999</v>
+      </c>
       <c r="L13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1575,7 +1593,9 @@
       <c r="J15" s="5" t="n">
         <v>0.1353</v>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="n">
+        <v>0.2162</v>
+      </c>
       <c r="L15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -1642,7 +1662,9 @@
       <c r="J16" s="5" t="n">
         <v>0.1778</v>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="n">
+        <v>0.2693</v>
+      </c>
       <c r="L16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -1725,7 +1747,9 @@
       <c r="J17" s="5" t="n">
         <v>0.2781</v>
       </c>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="n">
+        <v>0.1928</v>
+      </c>
       <c r="L17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1792,7 +1816,9 @@
       <c r="J18" s="5" t="n">
         <v>0.1147</v>
       </c>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="n">
+        <v>0.3103</v>
+      </c>
       <c r="L18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1859,7 +1885,9 @@
       <c r="J19" s="5" t="n">
         <v>0.2801</v>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="n">
+        <v>0.2607</v>
+      </c>
       <c r="L19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -1942,7 +1970,9 @@
       <c r="J20" s="5" t="n">
         <v>0.2431</v>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="n">
+        <v>0.2125</v>
+      </c>
       <c r="L20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2025,7 +2055,9 @@
       <c r="J21" s="5" t="n">
         <v>0.2403</v>
       </c>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="n">
+        <v>0.1922</v>
+      </c>
       <c r="L21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2108,7 +2140,9 @@
       <c r="J22" s="5" t="n">
         <v>0.5511</v>
       </c>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="n">
+        <v>0.5341</v>
+      </c>
       <c r="L22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2191,7 +2225,9 @@
       <c r="J23" s="5" t="n">
         <v>0.0614</v>
       </c>
-      <c r="K23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="n">
+        <v>0.1487</v>
+      </c>
       <c r="L23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2274,7 +2310,9 @@
       <c r="J24" s="5" t="n">
         <v>0.5639</v>
       </c>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="n">
+        <v>0.3973</v>
+      </c>
       <c r="L24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2357,7 +2395,9 @@
       <c r="J25" s="5" t="n">
         <v>0.0089</v>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="n">
+        <v>0.0169</v>
+      </c>
       <c r="L25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -2611,7 +2651,9 @@
       <c r="J29" s="5" t="n">
         <v>0.078</v>
       </c>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="K29" s="5" t="n">
+        <v>0.2905</v>
+      </c>
       <c r="L29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2694,7 +2736,9 @@
       <c r="J30" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="L30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2777,7 +2821,9 @@
       <c r="J31" s="5" t="n">
         <v>0.1153</v>
       </c>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="K31" s="5" t="n">
+        <v>0.036</v>
+      </c>
       <c r="L31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2860,7 +2906,9 @@
       <c r="J32" s="5" t="n">
         <v>0.0388</v>
       </c>
-      <c r="K32" s="5" t="inlineStr"/>
+      <c r="K32" s="5" t="n">
+        <v>0.2983</v>
+      </c>
       <c r="L32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2943,7 +2991,9 @@
       <c r="J33" s="5" t="n">
         <v>0.2694</v>
       </c>
-      <c r="K33" s="5" t="inlineStr"/>
+      <c r="K33" s="5" t="n">
+        <v>0.2848</v>
+      </c>
       <c r="L33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -3120,7 +3170,9 @@
       <c r="J36" s="5" t="n">
         <v>0.1146</v>
       </c>
-      <c r="K36" s="5" t="inlineStr"/>
+      <c r="K36" s="5" t="n">
+        <v>0.0936</v>
+      </c>
       <c r="L36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -3203,7 +3255,9 @@
       <c r="J37" s="5" t="n">
         <v>0.2365</v>
       </c>
-      <c r="K37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="n">
+        <v>0.2465</v>
+      </c>
       <c r="L37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -3349,7 +3403,9 @@
         <v>330</v>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="n">
+        <v>0.08939999999999999</v>
+      </c>
       <c r="L39" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -3430,7 +3486,9 @@
         <v>330</v>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
-      <c r="K40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="n">
+        <v>0.0813</v>
+      </c>
       <c r="L40" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -3513,7 +3571,9 @@
       <c r="J41" s="5" t="n">
         <v>0.1167</v>
       </c>
-      <c r="K41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="n">
+        <v>0.2803</v>
+      </c>
       <c r="L41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3596,7 +3656,9 @@
       <c r="J42" s="5" t="n">
         <v>0.2501</v>
       </c>
-      <c r="K42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="n">
+        <v>0.2261</v>
+      </c>
       <c r="L42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3677,7 +3739,9 @@
         <v>330</v>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
-      <c r="K43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="n">
+        <v>0.2674</v>
+      </c>
       <c r="L43" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3742,7 +3806,9 @@
         <v>330</v>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
-      <c r="K44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="n">
+        <v>0.2715</v>
+      </c>
       <c r="L44" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3809,7 +3875,9 @@
       <c r="J45" s="5" t="n">
         <v>0.0616</v>
       </c>
-      <c r="K45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="n">
+        <v>0.0283</v>
+      </c>
       <c r="L45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3892,7 +3960,9 @@
       <c r="J46" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="K46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="n">
+        <v>0.081</v>
+      </c>
       <c r="L46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3975,7 +4045,9 @@
       <c r="J47" s="5" t="n">
         <v>0.1883</v>
       </c>
-      <c r="K47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="n">
+        <v>0.1353</v>
+      </c>
       <c r="L47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -4042,7 +4114,9 @@
       <c r="J48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
-      <c r="K48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="n">
+        <v>0.0301</v>
+      </c>
       <c r="L48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -4123,7 +4197,9 @@
         <v>330</v>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
-      <c r="K49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="n">
+        <v>0.0216</v>
+      </c>
       <c r="L49" s="5" t="n">
         <v>0.158699742317549</v>
       </c>
@@ -4190,7 +4266,9 @@
       <c r="J50" s="5" t="n">
         <v>0.1969</v>
       </c>
-      <c r="K50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="n">
+        <v>0.1655</v>
+      </c>
       <c r="L50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -4251,7 +4329,9 @@
       <c r="J51" s="5" t="n">
         <v>0.0528</v>
       </c>
-      <c r="K51" s="5" t="inlineStr"/>
+      <c r="K51" s="5" t="n">
+        <v>0.0629</v>
+      </c>
       <c r="L51" s="5" t="inlineStr"/>
       <c r="M51" s="5" t="inlineStr"/>
       <c r="N51" s="5" t="n">
@@ -4308,7 +4388,9 @@
       <c r="J52" s="5" t="n">
         <v>0.1308</v>
       </c>
-      <c r="K52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="n">
+        <v>0.1312</v>
+      </c>
       <c r="L52" s="5" t="inlineStr"/>
       <c r="M52" s="5" t="inlineStr"/>
       <c r="N52" s="5" t="n">
@@ -4365,7 +4447,9 @@
       <c r="J53" s="5" t="n">
         <v>0.0143</v>
       </c>
-      <c r="K53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="n">
+        <v>0.0042</v>
+      </c>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr"/>
       <c r="N53" s="5" t="n">
@@ -4422,7 +4506,9 @@
       <c r="J54" s="5" t="n">
         <v>0.0265</v>
       </c>
-      <c r="K54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="n">
+        <v>0.0185</v>
+      </c>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
       <c r="N54" s="5" t="n">
@@ -4534,7 +4620,9 @@
       <c r="J56" s="5" t="n">
         <v>0.0066</v>
       </c>
-      <c r="K56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="n">
+        <v>0.0089</v>
+      </c>
       <c r="L56" s="5" t="inlineStr"/>
       <c r="M56" s="5" t="inlineStr"/>
       <c r="N56" s="5" t="n">
@@ -4589,7 +4677,9 @@
       </c>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="5" t="inlineStr"/>
-      <c r="K57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="n">
+        <v>0.0144</v>
+      </c>
       <c r="L57" s="5" t="inlineStr"/>
       <c r="M57" s="5" t="inlineStr"/>
       <c r="N57" s="5" t="n">
@@ -4644,7 +4734,9 @@
       </c>
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
-      <c r="K58" s="5" t="inlineStr"/>
+      <c r="K58" s="5" t="n">
+        <v>0.0219</v>
+      </c>
       <c r="L58" s="5" t="inlineStr"/>
       <c r="M58" s="5" t="inlineStr"/>
       <c r="N58" s="5" t="n">
@@ -4701,7 +4793,9 @@
       <c r="J59" s="5" t="n">
         <v>0.0298</v>
       </c>
-      <c r="K59" s="5" t="inlineStr"/>
+      <c r="K59" s="5" t="n">
+        <v>0.0184</v>
+      </c>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
       <c r="N59" s="5" t="n">
@@ -4813,7 +4907,9 @@
       <c r="J61" s="5" t="n">
         <v>0.0509</v>
       </c>
-      <c r="K61" s="5" t="inlineStr"/>
+      <c r="K61" s="5" t="n">
+        <v>0.019</v>
+      </c>
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
       <c r="N61" s="5" t="n">
@@ -4870,7 +4966,9 @@
       <c r="J62" s="5" t="n">
         <v>0.0168</v>
       </c>
-      <c r="K62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="n">
+        <v>0.0077</v>
+      </c>
       <c r="L62" s="5" t="inlineStr"/>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="n">
@@ -4927,7 +5025,9 @@
       <c r="J63" s="5" t="n">
         <v>0.055</v>
       </c>
-      <c r="K63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="n">
+        <v>0.009900000000000001</v>
+      </c>
       <c r="L63" s="5" t="inlineStr"/>
       <c r="M63" s="5" t="inlineStr"/>
       <c r="N63" s="5" t="n">
@@ -4984,7 +5084,9 @@
       <c r="J64" s="5" t="n">
         <v>0.0178</v>
       </c>
-      <c r="K64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="n">
+        <v>0.0214</v>
+      </c>
       <c r="L64" s="5" t="inlineStr"/>
       <c r="M64" s="5" t="inlineStr"/>
       <c r="N64" s="5" t="n">
@@ -5041,7 +5143,9 @@
       <c r="J65" s="5" t="n">
         <v>0.0134</v>
       </c>
-      <c r="K65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="n">
+        <v>0.0043</v>
+      </c>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
       <c r="N65" s="5" t="n">
@@ -5098,7 +5202,9 @@
       <c r="J66" s="5" t="n">
         <v>0.0056</v>
       </c>
-      <c r="K66" s="5" t="inlineStr"/>
+      <c r="K66" s="5" t="n">
+        <v>0.0102</v>
+      </c>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
       <c r="N66" s="5" t="n">
@@ -5155,7 +5261,9 @@
       <c r="J67" s="5" t="n">
         <v>0.064</v>
       </c>
-      <c r="K67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="n">
+        <v>0.07679999999999999</v>
+      </c>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
       <c r="N67" s="5" t="n">
@@ -5212,7 +5320,9 @@
       <c r="J68" s="5" t="n">
         <v>0.0002</v>
       </c>
-      <c r="K68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="n">
+        <v>0.0035</v>
+      </c>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
       <c r="N68" s="5" t="n">
@@ -5269,7 +5379,9 @@
       <c r="J69" s="5" t="n">
         <v>0.0573</v>
       </c>
-      <c r="K69" s="5" t="inlineStr"/>
+      <c r="K69" s="5" t="n">
+        <v>0.0549</v>
+      </c>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
       <c r="N69" s="5" t="n">
@@ -5326,7 +5438,9 @@
       <c r="J70" s="5" t="n">
         <v>0.0294</v>
       </c>
-      <c r="K70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="n">
+        <v>0.023</v>
+      </c>
       <c r="L70" s="5" t="inlineStr"/>
       <c r="M70" s="5" t="inlineStr"/>
       <c r="N70" s="5" t="n">
@@ -5514,7 +5628,9 @@
       <c r="E2" s="5" t="n">
         <v>0.1441</v>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="n">
+        <v>0.1695</v>
+      </c>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5596,7 +5712,9 @@
       <c r="E3" s="5" t="n">
         <v>0.128</v>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="n">
+        <v>0.078</v>
+      </c>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -5678,7 +5796,9 @@
       <c r="E4" s="5" t="n">
         <v>0.123</v>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>0.1001</v>
+      </c>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5760,7 +5880,9 @@
       <c r="E5" s="5" t="n">
         <v>0.1492</v>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="n">
+        <v>0.2117</v>
+      </c>
       <c r="G5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -5902,7 +6024,9 @@
       <c r="E7" s="5" t="n">
         <v>0.0292</v>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="n">
+        <v>0.0415</v>
+      </c>
       <c r="G7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -5968,7 +6092,9 @@
       <c r="E8" s="5" t="n">
         <v>0.0799</v>
       </c>
-      <c r="F8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="n">
+        <v>0.1689</v>
+      </c>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -6048,7 +6174,9 @@
         <v>0.8903</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="n">
+        <v>0.342</v>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
@@ -6110,7 +6238,9 @@
       <c r="E10" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="F10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="n">
+        <v>0.1175</v>
+      </c>
       <c r="G10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6302,7 +6432,9 @@
       <c r="E13" s="5" t="n">
         <v>0.3285</v>
       </c>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="n">
+        <v>0.3999</v>
+      </c>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6448,7 +6580,9 @@
       <c r="E15" s="5" t="n">
         <v>0.1353</v>
       </c>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="n">
+        <v>0.2162</v>
+      </c>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -6514,7 +6648,9 @@
       <c r="E16" s="5" t="n">
         <v>0.1778</v>
       </c>
-      <c r="F16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="n">
+        <v>0.2693</v>
+      </c>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -6596,7 +6732,9 @@
       <c r="E17" s="5" t="n">
         <v>0.2781</v>
       </c>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="n">
+        <v>0.1928</v>
+      </c>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6662,7 +6800,9 @@
       <c r="E18" s="5" t="n">
         <v>0.1147</v>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>0.3103</v>
+      </c>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6728,7 +6868,9 @@
       <c r="E19" s="5" t="n">
         <v>0.2801</v>
       </c>
-      <c r="F19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="n">
+        <v>0.2607</v>
+      </c>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -6810,7 +6952,9 @@
       <c r="E20" s="5" t="n">
         <v>0.2431</v>
       </c>
-      <c r="F20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="n">
+        <v>0.2125</v>
+      </c>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -6892,7 +7036,9 @@
       <c r="E21" s="5" t="n">
         <v>0.2403</v>
       </c>
-      <c r="F21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="n">
+        <v>0.1922</v>
+      </c>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -6974,7 +7120,9 @@
       <c r="E22" s="5" t="n">
         <v>0.5511</v>
       </c>
-      <c r="F22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="n">
+        <v>0.5341</v>
+      </c>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7056,7 +7204,9 @@
       <c r="E23" s="5" t="n">
         <v>0.0614</v>
       </c>
-      <c r="F23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="n">
+        <v>0.1487</v>
+      </c>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7138,7 +7288,9 @@
       <c r="E24" s="5" t="n">
         <v>0.5639</v>
       </c>
-      <c r="F24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="n">
+        <v>0.3973</v>
+      </c>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7220,7 +7372,9 @@
       <c r="E25" s="5" t="n">
         <v>0.0089</v>
       </c>
-      <c r="F25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="n">
+        <v>0.0169</v>
+      </c>
       <c r="G25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -7482,7 +7636,9 @@
       <c r="E29" s="5" t="n">
         <v>0.078</v>
       </c>
-      <c r="F29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="n">
+        <v>0.2905</v>
+      </c>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7564,7 +7720,9 @@
       <c r="E30" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="F30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7646,7 +7804,9 @@
       <c r="E31" s="5" t="n">
         <v>0.1153</v>
       </c>
-      <c r="F31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="n">
+        <v>0.036</v>
+      </c>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7728,7 +7888,9 @@
       <c r="E32" s="5" t="n">
         <v>0.0388</v>
       </c>
-      <c r="F32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="n">
+        <v>0.2983</v>
+      </c>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7810,7 +7972,9 @@
       <c r="E33" s="5" t="n">
         <v>0.2694</v>
       </c>
-      <c r="F33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="n">
+        <v>0.2848</v>
+      </c>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -7996,7 +8160,9 @@
       <c r="E36" s="5" t="n">
         <v>0.1146</v>
       </c>
-      <c r="F36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="n">
+        <v>0.0936</v>
+      </c>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -8078,7 +8244,9 @@
       <c r="E37" s="5" t="n">
         <v>0.2365</v>
       </c>
-      <c r="F37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="n">
+        <v>0.2465</v>
+      </c>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -8222,7 +8390,9 @@
         <v>0.9427</v>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="n">
+        <v>0.08939999999999999</v>
+      </c>
       <c r="G39" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -8302,7 +8472,9 @@
         <v>0.9427</v>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="n">
+        <v>0.0813</v>
+      </c>
       <c r="G40" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -8384,7 +8556,9 @@
       <c r="E41" s="5" t="n">
         <v>0.1167</v>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="n">
+        <v>0.2803</v>
+      </c>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8466,7 +8640,9 @@
       <c r="E42" s="5" t="n">
         <v>0.2501</v>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="n">
+        <v>0.2261</v>
+      </c>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8546,7 +8722,9 @@
         <v>0.8908</v>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="n">
+        <v>0.2674</v>
+      </c>
       <c r="G43" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8610,7 +8788,9 @@
         <v>0.8894</v>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
-      <c r="F44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="n">
+        <v>0.2715</v>
+      </c>
       <c r="G44" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8676,7 +8856,9 @@
       <c r="E45" s="5" t="n">
         <v>0.0616</v>
       </c>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="n">
+        <v>0.0283</v>
+      </c>
       <c r="G45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8758,7 +8940,9 @@
       <c r="E46" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="n">
+        <v>0.081</v>
+      </c>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8840,7 +9024,9 @@
       <c r="E47" s="5" t="n">
         <v>0.1883</v>
       </c>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="n">
+        <v>0.1353</v>
+      </c>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -8906,7 +9092,9 @@
       <c r="E48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
-      <c r="F48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="n">
+        <v>0.0301</v>
+      </c>
       <c r="G48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -8986,7 +9174,9 @@
         <v>0.955</v>
       </c>
       <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="n">
+        <v>0.0216</v>
+      </c>
       <c r="G49" s="5" t="n">
         <v>0.158699742317549</v>
       </c>
@@ -9052,7 +9242,9 @@
       <c r="E50" s="5" t="n">
         <v>0.1969</v>
       </c>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="n">
+        <v>0.1655</v>
+      </c>
       <c r="G50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -9118,7 +9310,9 @@
       <c r="E51" s="5" t="n">
         <v>0.0528</v>
       </c>
-      <c r="F51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="n">
+        <v>0.0629</v>
+      </c>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr"/>
@@ -9180,7 +9374,9 @@
       <c r="E52" s="5" t="n">
         <v>0.1308</v>
       </c>
-      <c r="F52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="n">
+        <v>0.1312</v>
+      </c>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
@@ -9242,7 +9438,9 @@
       <c r="E53" s="5" t="n">
         <v>0.0143</v>
       </c>
-      <c r="F53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="n">
+        <v>0.0042</v>
+      </c>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr"/>
@@ -9304,7 +9502,9 @@
       <c r="E54" s="5" t="n">
         <v>0.0265</v>
       </c>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="n">
+        <v>0.0185</v>
+      </c>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
@@ -9426,7 +9626,9 @@
       <c r="E56" s="5" t="n">
         <v>0.0066</v>
       </c>
-      <c r="F56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="n">
+        <v>0.0089</v>
+      </c>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
@@ -9486,7 +9688,9 @@
         <v>0.9644</v>
       </c>
       <c r="E57" s="5" t="inlineStr"/>
-      <c r="F57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="n">
+        <v>0.0144</v>
+      </c>
       <c r="G57" s="5" t="inlineStr"/>
       <c r="H57" s="5" t="inlineStr"/>
       <c r="I57" s="5" t="inlineStr"/>
@@ -9546,7 +9750,9 @@
         <v>0.9641999999999999</v>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
-      <c r="F58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="n">
+        <v>0.0219</v>
+      </c>
       <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr"/>
       <c r="I58" s="5" t="inlineStr"/>
@@ -9608,7 +9814,9 @@
       <c r="E59" s="5" t="n">
         <v>0.0298</v>
       </c>
-      <c r="F59" s="5" t="inlineStr"/>
+      <c r="F59" s="5" t="n">
+        <v>0.0184</v>
+      </c>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="5" t="inlineStr"/>
@@ -9730,7 +9938,9 @@
       <c r="E61" s="5" t="n">
         <v>0.0509</v>
       </c>
-      <c r="F61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="n">
+        <v>0.019</v>
+      </c>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr"/>
@@ -9792,7 +10002,9 @@
       <c r="E62" s="5" t="n">
         <v>0.0168</v>
       </c>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="n">
+        <v>0.0077</v>
+      </c>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr"/>
@@ -9854,7 +10066,9 @@
       <c r="E63" s="5" t="n">
         <v>0.055</v>
       </c>
-      <c r="F63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="n">
+        <v>0.009900000000000001</v>
+      </c>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
       <c r="I63" s="5" t="inlineStr"/>
@@ -9916,7 +10130,9 @@
       <c r="E64" s="5" t="n">
         <v>0.0178</v>
       </c>
-      <c r="F64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="n">
+        <v>0.0214</v>
+      </c>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr"/>
@@ -9978,7 +10194,9 @@
       <c r="E65" s="5" t="n">
         <v>0.0134</v>
       </c>
-      <c r="F65" s="5" t="inlineStr"/>
+      <c r="F65" s="5" t="n">
+        <v>0.0043</v>
+      </c>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr"/>
@@ -10040,7 +10258,9 @@
       <c r="E66" s="5" t="n">
         <v>0.0056</v>
       </c>
-      <c r="F66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="n">
+        <v>0.0102</v>
+      </c>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr"/>
@@ -10102,7 +10322,9 @@
       <c r="E67" s="5" t="n">
         <v>0.064</v>
       </c>
-      <c r="F67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="n">
+        <v>0.07679999999999999</v>
+      </c>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
       <c r="I67" s="5" t="inlineStr"/>
@@ -10164,7 +10386,9 @@
       <c r="E68" s="5" t="n">
         <v>0.0002</v>
       </c>
-      <c r="F68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="n">
+        <v>0.0035</v>
+      </c>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr"/>
@@ -10226,7 +10450,9 @@
       <c r="E69" s="5" t="n">
         <v>0.0573</v>
       </c>
-      <c r="F69" s="5" t="inlineStr"/>
+      <c r="F69" s="5" t="n">
+        <v>0.0549</v>
+      </c>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr"/>
@@ -10288,7 +10514,9 @@
       <c r="E70" s="5" t="n">
         <v>0.0294</v>
       </c>
-      <c r="F70" s="5" t="inlineStr"/>
+      <c r="F70" s="5" t="n">
+        <v>0.023</v>
+      </c>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr"/>

</xml_diff>